<commit_message>
Complete Exercise 4A and update Excel tables
</commit_message>
<xml_diff>
--- a/Mccutcheon_Ex3A_tables.xlsx
+++ b/Mccutcheon_Ex3A_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arionsaemccutcheon\Documents\DataAnalytics\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{6011A516-D566-45E3-BA60-E8CB7EE17502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{DCC2B178-1CC7-4382-98B0-282F28763764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{1660C6BD-3610-4D20-97F5-0B0768D6BFC6}"/>
+    <workbookView xWindow="312" yWindow="3576" windowWidth="11028" windowHeight="9960" firstSheet="2" activeTab="4" xr2:uid="{1660C6BD-3610-4D20-97F5-0B0768D6BFC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Owner" sheetId="1" r:id="rId1"/>
@@ -46,50 +46,26 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="26" uniqueCount="21">
-  <si>
-    <t>phoneNumber</t>
-  </si>
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="34" uniqueCount="32">
   <si>
     <t>email</t>
   </si>
   <si>
-    <t>ownerName</t>
-  </si>
-  <si>
     <t>ownerID</t>
   </si>
   <si>
     <t>dogID</t>
   </si>
   <si>
-    <t>dogName</t>
-  </si>
-  <si>
     <t>breed</t>
   </si>
   <si>
     <t>age</t>
   </si>
   <si>
-    <t>medicalHistory</t>
-  </si>
-  <si>
     <t>walkID</t>
   </si>
   <si>
-    <t>walkDate</t>
-  </si>
-  <si>
-    <t>startTime</t>
-  </si>
-  <si>
-    <t>endTime</t>
-  </si>
-  <si>
-    <t>walkDuration</t>
-  </si>
-  <si>
     <t>notes</t>
   </si>
   <si>
@@ -109,16 +85,85 @@
   </si>
   <si>
     <t>dateCharged</t>
+  </si>
+  <si>
+    <t>Joe Blue</t>
+  </si>
+  <si>
+    <t>(929)123-4567</t>
+  </si>
+  <si>
+    <t>Jblue@gmail.com</t>
+  </si>
+  <si>
+    <t>owner_id</t>
+  </si>
+  <si>
+    <t>owner_name</t>
+  </si>
+  <si>
+    <t>phone_number</t>
+  </si>
+  <si>
+    <t>dog_id</t>
+  </si>
+  <si>
+    <t>dog_name</t>
+  </si>
+  <si>
+    <t>medical_history</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poodle </t>
+  </si>
+  <si>
+    <t xml:space="preserve">None </t>
+  </si>
+  <si>
+    <t>walk_id</t>
+  </si>
+  <si>
+    <t>walk_date</t>
+  </si>
+  <si>
+    <t>start_time</t>
+  </si>
+  <si>
+    <t>end_time</t>
+  </si>
+  <si>
+    <t>walk_duration</t>
+  </si>
+  <si>
+    <t>walk went well</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credit </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="167" formatCode="[h]:mm:ss;@"/>
+    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -165,17 +210,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -508,61 +560,96 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D812DFAB-3C99-4E9F-844A-D61C2E8F7244}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" t="s">
-        <v>1</v>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{FCF2CC9E-1281-48DE-A1DF-502A357BAA88}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75C4CD00-7E0E-469C-A0D9-D83559138883}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="6.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" t="s">
-        <v>7</v>
-      </c>
       <c r="F1" t="s">
-        <v>8</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -572,35 +659,52 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{164EE6E9-E79A-4A1D-B769-855F9C368E7A}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="B1" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="D1" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="E1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F1" t="s">
-        <v>14</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B2" s="8" t="d">
+        <v>2026-10-27</v>
+      </c>
+      <c r="C2" s="7" t="d">
+        <v>PT8H0M0.000S</v>
+      </c>
+      <c r="D2" s="7" t="d">
+        <v>PT8H30M0.000S</v>
+      </c>
+      <c r="E2">
+        <v>30</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -610,7 +714,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3364477D-A5CC-4521-B53D-E66E4F7A263F}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.88671875" style="3"/>
@@ -618,16 +722,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1</v>
+      </c>
+      <c r="C2" s="9" t="d">
+        <v>07:54:59.99999999999946525</v>
+      </c>
+      <c r="D2" s="9" t="d">
+        <v>08:35:00.00000000000053475</v>
       </c>
     </row>
   </sheetData>
@@ -637,7 +755,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9284E0F1-CB59-4D08-8951-76BE5E792CE3}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.5546875" style="1" bestFit="1" customWidth="1"/>
@@ -650,22 +768,39 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F1" t="s">
-        <v>20</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="6" t="d">
+        <v>2026-10-27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>